<commit_message>
Table 1: integer ages, severity column with instruments and results
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018JDGfvcxTbt2jG2mX2x2rD
</commit_message>
<xml_diff>
--- a/表1_文献信息编码表.xlsx
+++ b/表1_文献信息编码表.xlsx
@@ -471,8 +471,8 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>8.8～11.2</t>
+          <t>8～11</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -743,12 +743,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>3.8～4.2</t>
+          <t>3～4</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>轻中度、重度</t>
+          <t>CARS 36～39 轻中度、重度</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -801,12 +801,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>2.7～3.7</t>
+          <t>2～3</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>重度</t>
+          <t>CARS 39.5～45 重度</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>4～4.2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>重度</t>
+          <t>CARS 重度；GARS 一般可能、很可能</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GARS-3 很可能</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -975,12 +975,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>7.1～11.8</t>
+          <t>7～11</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV-TR 诊断</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>10.3～12.4</t>
+          <t>10～12</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1091,12 +1091,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>3.9～5.6</t>
+          <t>3～5</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV 诊断</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>7.2～9.2</t>
+          <t>7～9</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV 诊断</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>7.8～12.5</t>
+          <t>7～12</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>4.5～5.2</t>
+          <t>4～5</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1323,12 +1323,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>3～3.9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ADOS 孤独症范围</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>6.3～8.8</t>
+          <t>6～8</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-5 诊断</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>5～12.1</t>
+          <t>5～12</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>轻中度</t>
+          <t>CARS 31～35.5 轻中度</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1671,12 +1671,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>7.5～10.5</t>
+          <t>7～10</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>轻中度</t>
+          <t>CARS 33.5～36.5 轻中度</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>6.5～7</t>
+          <t>6～7</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>轻中度、重度</t>
+          <t>CARS 31～44 轻中度、重度</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1787,12 +1787,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>3.8～5.2</t>
+          <t>3～5</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GARS-2 可能、很可能</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>10.6～11.7</t>
+          <t>10～11</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GARS-2、ASDS 很可能</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>4.2～4.4</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>5～5.8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GARS-2 很可能；ASRS 升高</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>7.2～9.5</t>
+          <t>7～9</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ASRS 升高</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2309,12 +2309,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>6.5～9.2</t>
+          <t>6～9</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV-TR 诊断；GARS 一般可能；GADS 很可能</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV-TR 诊断</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2425,12 +2425,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>4～11.2</t>
+          <t>4～11</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>轻中度、重度</t>
+          <t>CARS 33.5～41.5 轻中度、重度</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>轻中度</t>
+          <t>原文说明 轻中度</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV 诊断</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2599,12 +2599,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>6.5～12.2</t>
+          <t>6～12</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>轻中度、重度</t>
+          <t>CARS 30～39.5 轻中度、重度</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2657,12 +2657,12 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>4～5.5</t>
+          <t>4～5</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DSM-IV 诊断</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>轻中度</t>
+          <t>CARS 轻中度</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -2812,10 +2812,10 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="48" customHeight="1">
+    <row r="42" ht="90" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>注：—表示原文未报告。示范者、干预方式、单次时长等一项含多个取值的，表示该研究不同儿童或不同阶段的编码不同。Boudreau，2013原文只报告样本年龄范围，且有1名被试未报告性别；Buggey，2016、Buggey，2012分别有1名、1名被试未报告孤独症程度；Murphy，2018、Williamson，2013原文仅报告年级（分别为5～6年级、6年级）。同一第一作者同年发表的文献以a、b区分。</t>
+          <t>注：—表示原文未报告。孤独症程度一栏列出原文报告的诊断标准或评估工具及其结果，其中轻中度、重度依据CARS分数或原文说明判定（见2.2.2），其余仅为诊断信息，不参与程度分组。DSM为精神障碍诊断与统计手册；CARS为儿童孤独症评定量表；GARS为吉列姆孤独症评定量表，GARS-2、GARS-3分别为第二、三版；ADOS为孤独症诊断观察量表；ASRS为孤独症谱系评定量表；ASDS为阿斯伯格综合征诊断量表；GADS为吉列姆阿斯伯格障碍量表。示范者、干预方式、单次时长等一项含多个取值的，表示该研究不同儿童或不同阶段的编码不同。年龄按实足年龄取整。Boudreau，2013原文只报告样本年龄范围，且有1名被试未报告性别；Buggey，2016、Buggey，2012各有1名被试无可判断程度的信息；Murphy，2018、Williamson，2013原文仅报告年级（分别为5～6年级、6年级）。同一第一作者同年发表的文献以a、b区分。</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2844,6 +2844,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2882,6 +2883,11 @@
           <t>作者年份来源</t>
         </is>
       </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>程度一栏需核对</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2907,7 +2913,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2915,6 +2921,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2948,6 +2955,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2973,7 +2981,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2981,6 +2989,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3006,7 +3015,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3014,6 +3023,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3039,7 +3049,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3047,6 +3057,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3072,7 +3083,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3080,6 +3091,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3105,7 +3117,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3113,6 +3125,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3138,7 +3151,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3146,6 +3159,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3171,7 +3185,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3179,6 +3193,7 @@
           <t>原文PDF首页</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -3204,12 +3219,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>WWC评级记录</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>原文写作“DSM-V”，但该文发表于2005年（DSM-5于2013年出版），表中按DSM-IV填写，请核对原文</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3257,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3245,6 +3265,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3270,7 +3291,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3278,6 +3299,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -3303,12 +3325,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>原文PDF（文件名）</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PDF中文字无法提取，未能读取被试诊断信息，暂填“—”，请核对原文</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3363,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3344,6 +3371,7 @@
           <t>原文PDF首页（Huan Li等，2025，IJDDE 72(2)，2024年在线）</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3369,7 +3397,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3377,6 +3405,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -3402,7 +3431,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3410,6 +3439,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -3435,7 +3465,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3443,6 +3473,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3476,6 +3507,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3509,6 +3541,7 @@
           <t>原文PDF首页（JABA 2004）</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3534,7 +3567,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3542,6 +3575,7 @@
           <t>原文PDF自注2004b（EJBA）</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3567,7 +3601,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3575,6 +3609,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3600,7 +3635,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3608,6 +3643,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3633,7 +3669,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3641,6 +3677,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3666,7 +3703,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3674,6 +3711,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3699,7 +3737,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3707,6 +3745,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3732,7 +3771,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3740,6 +3779,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3765,7 +3805,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3773,6 +3813,7 @@
           <t>原文PDF首页（ETC 2017）</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3798,7 +3839,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3806,6 +3847,7 @@
           <t>WWC记录作2016（在线年份）；按参考文献表采用2017年卷期</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3831,7 +3873,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3839,6 +3881,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3864,7 +3907,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3872,6 +3915,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3897,7 +3941,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3905,6 +3949,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3930,7 +3975,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3938,6 +3983,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3963,7 +4009,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3971,6 +4017,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3996,7 +4043,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -4004,6 +4051,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -4029,7 +4077,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4037,6 +4085,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4062,7 +4111,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4070,6 +4119,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4095,7 +4145,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -4103,6 +4153,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4136,6 +4187,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4161,7 +4213,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>按K分组表“年龄依据”列实际年龄取最小～最大</t>
+          <t>按K分组表“年龄依据”列实际年龄取整后取最小～最大</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -4169,6 +4221,7 @@
           <t>WWC评级记录</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">

</xml_diff>